<commit_message>
Intial extraction of fiel pig slurry
Inital extraction of field pig slurry from the raw picarro files
</commit_message>
<xml_diff>
--- a/Field-trails/Pig-Slurry 2025-11-05/DFC overview pig.xlsx
+++ b/Field-trails/Pig-Slurry 2025-11-05/DFC overview pig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\Pig-Slurry 2025-11-05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00DA8F7-FD18-4B4F-844E-EEF499DD54A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999721EB-CC28-4CD8-9604-A76F428A2C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,9 +88,6 @@
     <t>H2SO4</t>
   </si>
   <si>
-    <t>No acid</t>
-  </si>
-  <si>
     <t>AA</t>
   </si>
   <si>
@@ -157,6 +154,9 @@
   </si>
   <si>
     <t>emperical correction factor</t>
+  </si>
+  <si>
+    <t>RAW</t>
   </si>
 </sst>
 </file>
@@ -519,19 +519,19 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
-      </c>
-      <c r="L1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -561,10 +561,10 @@
         <v>3</v>
       </c>
       <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
         <v>29</v>
-      </c>
-      <c r="L2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -617,7 +617,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -641,7 +641,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -686,7 +686,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -755,7 +755,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -764,7 +764,7 @@
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F11">
         <v>129.4</v>
@@ -785,7 +785,7 @@
         <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F12">
         <v>121.4</v>
@@ -800,7 +800,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13">
         <v>12</v>
@@ -809,7 +809,7 @@
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13">
         <v>124.3</v>
@@ -824,7 +824,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -854,7 +854,7 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F15">
         <v>126.5</v>
@@ -869,7 +869,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16">
         <v>15</v>
@@ -878,7 +878,7 @@
         <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F16">
         <v>143.1</v>
@@ -893,7 +893,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17">
         <v>16</v>
@@ -923,7 +923,7 @@
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F18">
         <v>135.30000000000001</v>
@@ -938,7 +938,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19">
         <v>18</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20">
         <v>19</v>

</xml_diff>